<commit_message>
docs: streamline README and DAX documentation to pure institutional architecture
</commit_message>
<xml_diff>
--- a/reports/Exception_Report_2026-07-24.xlsx
+++ b/reports/Exception_Report_2026-07-24.xlsx
@@ -599,7 +599,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Valuation Date: 2026-07-24  |  Generated: 2026-09-29 17:28:59  |  Governance: UBS Group Finance / Product Control</t>
+          <t>Valuation Date: 2026-07-24  |  Generated: 2026-09-29 18:11:42  |  Governance: UBS Group Finance / Product Control</t>
         </is>
       </c>
     </row>
@@ -708,7 +708,7 @@
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="10" t="n">
-        <v>165</v>
+        <v>39</v>
       </c>
       <c r="B9" s="10" t="inlineStr">
         <is>
@@ -757,7 +757,7 @@
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="10" t="n">
-        <v>167</v>
+        <v>41</v>
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
@@ -806,7 +806,7 @@
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="10" t="n">
-        <v>166</v>
+        <v>40</v>
       </c>
       <c r="B11" s="10" t="inlineStr">
         <is>
@@ -855,7 +855,7 @@
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="10" t="n">
-        <v>168</v>
+        <v>42</v>
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>

</xml_diff>